<commit_message>
Rebuild curtailment via NEMOSIS + refresh outputs with June 2025 data
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/TAS_curtailment.xlsx
+++ b/outputs/TAS_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -481,6 +481,8 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,65 +533,75 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Actual FY23-24</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Actual FY24-25</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>ELI Near Term</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ELI Med Term</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>FY24-25</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>FY25-26</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>FY26-27 (Draft)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Curt FY1</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Curt FY2</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Curt FY3</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Curt Avg</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Offl FY1</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Offl FY2</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Offl FY3</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Offl Avg</t>
         </is>
@@ -631,25 +643,31 @@
         <v>148</v>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr"/>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="n">
+      <c r="J2" s="5" t="n">
+        <v>0.0007606441489553806</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>0.001353761908430395</v>
+      </c>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="n">
         <v>0.9908</v>
       </c>
-      <c r="M2" s="5" t="n">
+      <c r="O2" s="5" t="n">
         <v>0.9923999999999999</v>
       </c>
-      <c r="N2" s="5" t="n">
+      <c r="P2" s="5" t="n">
         <v>0.998</v>
       </c>
-      <c r="O2" s="6" t="inlineStr"/>
-      <c r="P2" s="6" t="inlineStr"/>
       <c r="Q2" s="6" t="inlineStr"/>
       <c r="R2" s="6" t="inlineStr"/>
       <c r="S2" s="6" t="inlineStr"/>
       <c r="T2" s="6" t="inlineStr"/>
       <c r="U2" s="6" t="inlineStr"/>
       <c r="V2" s="6" t="inlineStr"/>
+      <c r="W2" s="6" t="inlineStr"/>
+      <c r="X2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -687,25 +705,31 @@
         <v>110</v>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="n">
+      <c r="J3" s="5" t="n">
+        <v>0.003277580990602602</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0.001248395140656555</v>
+      </c>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
+      <c r="N3" s="5" t="n">
         <v>0.9473</v>
       </c>
-      <c r="M3" s="5" t="n">
+      <c r="O3" s="5" t="n">
         <v>0.9555</v>
       </c>
-      <c r="N3" s="5" t="n">
+      <c r="P3" s="5" t="n">
         <v>0.9611</v>
       </c>
-      <c r="O3" s="6" t="inlineStr"/>
-      <c r="P3" s="6" t="inlineStr"/>
       <c r="Q3" s="6" t="inlineStr"/>
       <c r="R3" s="6" t="inlineStr"/>
       <c r="S3" s="6" t="inlineStr"/>
       <c r="T3" s="6" t="inlineStr"/>
       <c r="U3" s="6" t="inlineStr"/>
       <c r="V3" s="6" t="inlineStr"/>
+      <c r="W3" s="6" t="inlineStr"/>
+      <c r="X3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -743,25 +767,31 @@
         <v>168</v>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="n">
+      <c r="J4" s="5" t="n">
+        <v>0.01315360223580064</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0.01356352485911394</v>
+      </c>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="n">
         <v>0.9199000000000001</v>
       </c>
-      <c r="M4" s="5" t="n">
+      <c r="O4" s="5" t="n">
         <v>0.9101</v>
       </c>
-      <c r="N4" s="5" t="n">
+      <c r="P4" s="5" t="n">
         <v>0.9125</v>
       </c>
-      <c r="O4" s="6" t="inlineStr"/>
-      <c r="P4" s="6" t="inlineStr"/>
       <c r="Q4" s="6" t="inlineStr"/>
       <c r="R4" s="6" t="inlineStr"/>
       <c r="S4" s="6" t="inlineStr"/>
       <c r="T4" s="6" t="inlineStr"/>
       <c r="U4" s="6" t="inlineStr"/>
       <c r="V4" s="6" t="inlineStr"/>
+      <c r="W4" s="6" t="inlineStr"/>
+      <c r="X4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -801,23 +831,25 @@
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="n">
         <v>0.8951</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="O5" s="5" t="n">
         <v>0.9224</v>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="P5" s="5" t="n">
         <v>0.9324</v>
       </c>
-      <c r="O5" s="6" t="inlineStr"/>
-      <c r="P5" s="6" t="inlineStr"/>
       <c r="Q5" s="6" t="inlineStr"/>
       <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="6" t="inlineStr"/>
       <c r="T5" s="6" t="inlineStr"/>
       <c r="U5" s="6" t="inlineStr"/>
       <c r="V5" s="6" t="inlineStr"/>
+      <c r="W5" s="6" t="inlineStr"/>
+      <c r="X5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -830,7 +862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -854,6 +886,8 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -884,80 +918,90 @@
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
+          <t>CURTAILMENT_ACTUAL_FY23-24</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>CURTAILMENT_ACTUAL_FY24-25</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
           <t>ELI_CURTAILMENT_NEAR</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>ELI_CURTAILMENT_MED</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY1</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY1_LABEL</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY2</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY2_LABEL</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY3</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_FY3_LABEL</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>ISP_CURTAILMENT_AVG</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY1</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY1_LABEL</t>
         </is>
       </c>
-      <c r="Q1" s="7" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY2</t>
         </is>
       </c>
-      <c r="R1" s="7" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY2_LABEL</t>
         </is>
       </c>
-      <c r="S1" s="7" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY3</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_FY3_LABEL</t>
         </is>
       </c>
-      <c r="U1" s="7" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_AVG</t>
         </is>
@@ -983,46 +1027,52 @@
       <c r="E2" s="5" t="n">
         <v>0.998</v>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="n">
+        <v>0.0007606441489553806</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.001353761908430395</v>
+      </c>
       <c r="H2" s="5" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr"/>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr"/>
-      <c r="P2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="P2" s="5" t="inlineStr"/>
       <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr"/>
       <c r="T2" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr"/>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr"/>
+      <c r="W2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1044,46 +1094,52 @@
       <c r="E3" s="5" t="n">
         <v>0.9611</v>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="n">
+        <v>0.003277580990602602</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.001248395140656555</v>
+      </c>
       <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="5" t="inlineStr"/>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr"/>
       <c r="M3" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr"/>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr"/>
-      <c r="P3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr"/>
       <c r="T3" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr"/>
+      <c r="W3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -1105,46 +1161,52 @@
       <c r="E4" s="5" t="n">
         <v>0.9125</v>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>0.01315360223580064</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.01356352485911394</v>
+      </c>
       <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr"/>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr"/>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr"/>
       <c r="T4" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr"/>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr"/>
+      <c r="W4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1169,43 +1231,45 @@
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="inlineStr"/>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>26-27</t>
+          <t>25-26</t>
         </is>
       </c>
       <c r="S5" s="5" t="inlineStr"/>
       <c r="T5" s="5" t="inlineStr">
         <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="U5" s="5" t="inlineStr"/>
+      <c r="W5" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C5">
@@ -1436,6 +1500,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="V2:V5">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W2:W5">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Source actual curtailment from credit dashboard instead of running NEMOSIS
The renewable dashboard was re-deriving 2 FYs of SCADA + DISPATCHLOAD via
NEMOSIS every run, which duplicated work the credit dashboard already does
monthly and blew the GitHub runner's memory on full refresh.

Now fetches the credit dashboard's published curtailment_by_fy.csv (per-DUID
per-FY rollup, generation-weighted). NEMOSIS dependency, nemosis_cache
symlink, download_curtailment.py and the --skip-scada / August-1 full-refresh
branches are all removed. Monthly cron moves to the 20th so credit's 18th run
has published a fresh rollup by the time we fetch it.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/TAS_curtailment.xlsx
+++ b/outputs/TAS_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -82,9 +82,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -456,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -475,14 +472,6 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,46 +555,6 @@
           <t>FY26-27 (Draft)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY1</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY2</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY3</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Curt Avg</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY1</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY2</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY3</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Offl Avg</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -644,10 +593,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="5" t="n">
-        <v>0.0007606441489553806</v>
+        <v>0.0051</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>0.001353761908430395</v>
+        <v>0.0068</v>
       </c>
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
@@ -660,14 +609,6 @@
       <c r="P2" s="5" t="n">
         <v>0.998</v>
       </c>
-      <c r="Q2" s="6" t="inlineStr"/>
-      <c r="R2" s="6" t="inlineStr"/>
-      <c r="S2" s="6" t="inlineStr"/>
-      <c r="T2" s="6" t="inlineStr"/>
-      <c r="U2" s="6" t="inlineStr"/>
-      <c r="V2" s="6" t="inlineStr"/>
-      <c r="W2" s="6" t="inlineStr"/>
-      <c r="X2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -706,10 +647,10 @@
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="5" t="n">
-        <v>0.003277580990602602</v>
+        <v>0.007</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.001248395140656555</v>
+        <v>0.0033</v>
       </c>
       <c r="L3" s="5" t="inlineStr"/>
       <c r="M3" s="5" t="inlineStr"/>
@@ -722,14 +663,6 @@
       <c r="P3" s="5" t="n">
         <v>0.9611</v>
       </c>
-      <c r="Q3" s="6" t="inlineStr"/>
-      <c r="R3" s="6" t="inlineStr"/>
-      <c r="S3" s="6" t="inlineStr"/>
-      <c r="T3" s="6" t="inlineStr"/>
-      <c r="U3" s="6" t="inlineStr"/>
-      <c r="V3" s="6" t="inlineStr"/>
-      <c r="W3" s="6" t="inlineStr"/>
-      <c r="X3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -768,10 +701,10 @@
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="5" t="n">
-        <v>0.01315360223580064</v>
+        <v>0.013</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>0.01356352485911394</v>
+        <v>0.0135</v>
       </c>
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
@@ -784,14 +717,6 @@
       <c r="P4" s="5" t="n">
         <v>0.9125</v>
       </c>
-      <c r="Q4" s="6" t="inlineStr"/>
-      <c r="R4" s="6" t="inlineStr"/>
-      <c r="S4" s="6" t="inlineStr"/>
-      <c r="T4" s="6" t="inlineStr"/>
-      <c r="U4" s="6" t="inlineStr"/>
-      <c r="V4" s="6" t="inlineStr"/>
-      <c r="W4" s="6" t="inlineStr"/>
-      <c r="X4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -842,14 +767,6 @@
       <c r="P5" s="5" t="n">
         <v>0.9324</v>
       </c>
-      <c r="Q5" s="6" t="inlineStr"/>
-      <c r="R5" s="6" t="inlineStr"/>
-      <c r="S5" s="6" t="inlineStr"/>
-      <c r="T5" s="6" t="inlineStr"/>
-      <c r="U5" s="6" t="inlineStr"/>
-      <c r="V5" s="6" t="inlineStr"/>
-      <c r="W5" s="6" t="inlineStr"/>
-      <c r="X5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -862,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -874,146 +791,62 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>DUID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Fuel</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>MLF_FY24-25</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>MLF_FY25-26</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>MLF_FY26-27 (Draft)</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>CURTAILMENT_ACTUAL_FY23-24</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>CURTAILMENT_ACTUAL_FY24-25</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>ELI_CURTAILMENT_NEAR</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>ELI_CURTAILMENT_MED</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY1</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY1_LABEL</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY2</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY2_LABEL</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY3</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY3_LABEL</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_AVG</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY1</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY1_LABEL</t>
-        </is>
-      </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY2</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY2_LABEL</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY3</t>
-        </is>
-      </c>
-      <c r="V1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY3_LABEL</t>
-        </is>
-      </c>
-      <c r="W1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_AVG</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>CTHLWF1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -1028,59 +861,21 @@
         <v>0.998</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.0007606441489553806</v>
+        <v>0.0051</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.001353761908430395</v>
+        <v>0.0068</v>
       </c>
       <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr"/>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="S2" s="5" t="inlineStr"/>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="U2" s="5" t="inlineStr"/>
-      <c r="V2" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>GRANWF1</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -1095,59 +890,21 @@
         <v>0.9611</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.003277580990602602</v>
+        <v>0.007</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>0.001248395140656555</v>
+        <v>0.0033</v>
       </c>
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="S3" s="5" t="inlineStr"/>
-      <c r="T3" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="W3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>MUSSELR1</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -1162,59 +919,21 @@
         <v>0.9125</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.01315360223580064</v>
+        <v>0.013</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0.01356352485911394</v>
+        <v>0.0135</v>
       </c>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="U4" s="5" t="inlineStr"/>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="W4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>WOOLNTH1</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -1232,44 +951,6 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="S5" s="5" t="inlineStr"/>
-      <c r="T5" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="U5" s="5" t="inlineStr"/>
-      <c r="V5" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="W5" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C5">
@@ -1356,174 +1037,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J5">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K5">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L5">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M5">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N5">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O5">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P5">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q5">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R5">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S5">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T5">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U5">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V5">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W5">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update FY26-27 MLFs from draft to final
Re-run after MLF Tracker ingested AEMO's published final Excel.
MLF_FY26-27 (Draft) replaced by MLF_FY26-27 with genuine final values.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/TAS_curtailment.xlsx
+++ b/outputs/TAS_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:W5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,6 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,55 +552,50 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>FY24-25</t>
+          <t>FY25-26</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>FY25-26</t>
+          <t>FY26-27</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>FY26-27 (Draft)</t>
+          <t>Curt FY1</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Curt FY1</t>
+          <t>Curt FY2</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Curt FY2</t>
+          <t>Curt FY3</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Curt FY3</t>
+          <t>Curt Avg</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Curt Avg</t>
+          <t>Offl FY1</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Offl FY1</t>
+          <t>Offl FY2</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Offl FY2</t>
+          <t>Offl FY3</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY3</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Offl Avg</t>
         </is>
@@ -652,14 +646,12 @@
       <c r="L2" s="5" t="inlineStr"/>
       <c r="M2" s="5" t="inlineStr"/>
       <c r="N2" s="5" t="n">
-        <v>0.9908</v>
+        <v>0.9923999999999999</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>0.9923999999999999</v>
-      </c>
-      <c r="P2" s="5" t="n">
-        <v>0.998</v>
-      </c>
+        <v>1.0088</v>
+      </c>
+      <c r="P2" s="6" t="inlineStr"/>
       <c r="Q2" s="6" t="inlineStr"/>
       <c r="R2" s="6" t="inlineStr"/>
       <c r="S2" s="6" t="inlineStr"/>
@@ -667,7 +659,6 @@
       <c r="U2" s="6" t="inlineStr"/>
       <c r="V2" s="6" t="inlineStr"/>
       <c r="W2" s="6" t="inlineStr"/>
-      <c r="X2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -714,14 +705,12 @@
       <c r="L3" s="5" t="inlineStr"/>
       <c r="M3" s="5" t="inlineStr"/>
       <c r="N3" s="5" t="n">
-        <v>0.9473</v>
+        <v>0.9555</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>0.9555</v>
-      </c>
-      <c r="P3" s="5" t="n">
-        <v>0.9611</v>
-      </c>
+        <v>0.9688</v>
+      </c>
+      <c r="P3" s="6" t="inlineStr"/>
       <c r="Q3" s="6" t="inlineStr"/>
       <c r="R3" s="6" t="inlineStr"/>
       <c r="S3" s="6" t="inlineStr"/>
@@ -729,7 +718,6 @@
       <c r="U3" s="6" t="inlineStr"/>
       <c r="V3" s="6" t="inlineStr"/>
       <c r="W3" s="6" t="inlineStr"/>
-      <c r="X3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -776,14 +764,12 @@
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr"/>
       <c r="N4" s="5" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.9101</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>0.9101</v>
-      </c>
-      <c r="P4" s="5" t="n">
-        <v>0.9125</v>
-      </c>
+        <v>0.9188</v>
+      </c>
+      <c r="P4" s="6" t="inlineStr"/>
       <c r="Q4" s="6" t="inlineStr"/>
       <c r="R4" s="6" t="inlineStr"/>
       <c r="S4" s="6" t="inlineStr"/>
@@ -791,7 +777,6 @@
       <c r="U4" s="6" t="inlineStr"/>
       <c r="V4" s="6" t="inlineStr"/>
       <c r="W4" s="6" t="inlineStr"/>
-      <c r="X4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -834,14 +819,12 @@
       <c r="L5" s="5" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr"/>
       <c r="N5" s="5" t="n">
-        <v>0.8951</v>
+        <v>0.9224</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>0.9224</v>
-      </c>
-      <c r="P5" s="5" t="n">
-        <v>0.9324</v>
-      </c>
+        <v>0.9371</v>
+      </c>
+      <c r="P5" s="6" t="inlineStr"/>
       <c r="Q5" s="6" t="inlineStr"/>
       <c r="R5" s="6" t="inlineStr"/>
       <c r="S5" s="6" t="inlineStr"/>
@@ -849,7 +832,6 @@
       <c r="U5" s="6" t="inlineStr"/>
       <c r="V5" s="6" t="inlineStr"/>
       <c r="W5" s="6" t="inlineStr"/>
-      <c r="X5" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -862,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -887,7 +869,6 @@
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -903,105 +884,100 @@
       </c>
       <c r="C1" s="7" t="inlineStr">
         <is>
-          <t>MLF_FY24-25</t>
+          <t>MLF_FY25-26</t>
         </is>
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
-          <t>MLF_FY25-26</t>
+          <t>MLF_FY26-27</t>
         </is>
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>MLF_FY26-27 (Draft)</t>
+          <t>CURTAILMENT_ACTUAL_FY23-24</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY23-24</t>
+          <t>CURTAILMENT_ACTUAL_FY24-25</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY24-25</t>
+          <t>ELI_CURTAILMENT_NEAR</t>
         </is>
       </c>
       <c r="H1" s="7" t="inlineStr">
         <is>
-          <t>ELI_CURTAILMENT_NEAR</t>
+          <t>ELI_CURTAILMENT_MED</t>
         </is>
       </c>
       <c r="I1" s="7" t="inlineStr">
         <is>
-          <t>ELI_CURTAILMENT_MED</t>
+          <t>ISP_CURTAILMENT_FY1</t>
         </is>
       </c>
       <c r="J1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY1</t>
+          <t>ISP_CURTAILMENT_FY1_LABEL</t>
         </is>
       </c>
       <c r="K1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY1_LABEL</t>
+          <t>ISP_CURTAILMENT_FY2</t>
         </is>
       </c>
       <c r="L1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY2</t>
+          <t>ISP_CURTAILMENT_FY2_LABEL</t>
         </is>
       </c>
       <c r="M1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY2_LABEL</t>
+          <t>ISP_CURTAILMENT_FY3</t>
         </is>
       </c>
       <c r="N1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY3</t>
+          <t>ISP_CURTAILMENT_FY3_LABEL</t>
         </is>
       </c>
       <c r="O1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_FY3_LABEL</t>
+          <t>ISP_CURTAILMENT_AVG</t>
         </is>
       </c>
       <c r="P1" s="7" t="inlineStr">
         <is>
-          <t>ISP_CURTAILMENT_AVG</t>
+          <t>ISP_OFFLOADING_FY1</t>
         </is>
       </c>
       <c r="Q1" s="7" t="inlineStr">
         <is>
-          <t>ISP_OFFLOADING_FY1</t>
+          <t>ISP_OFFLOADING_FY1_LABEL</t>
         </is>
       </c>
       <c r="R1" s="7" t="inlineStr">
         <is>
-          <t>ISP_OFFLOADING_FY1_LABEL</t>
+          <t>ISP_OFFLOADING_FY2</t>
         </is>
       </c>
       <c r="S1" s="7" t="inlineStr">
         <is>
-          <t>ISP_OFFLOADING_FY2</t>
+          <t>ISP_OFFLOADING_FY2_LABEL</t>
         </is>
       </c>
       <c r="T1" s="7" t="inlineStr">
         <is>
-          <t>ISP_OFFLOADING_FY2_LABEL</t>
+          <t>ISP_OFFLOADING_FY3</t>
         </is>
       </c>
       <c r="U1" s="7" t="inlineStr">
         <is>
-          <t>ISP_OFFLOADING_FY3</t>
+          <t>ISP_OFFLOADING_FY3_LABEL</t>
         </is>
       </c>
       <c r="V1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY3_LABEL</t>
-        </is>
-      </c>
-      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>ISP_OFFLOADING_AVG</t>
         </is>
@@ -1019,60 +995,57 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>0.9908</v>
+        <v>0.9923999999999999</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0.9923999999999999</v>
+        <v>1.0088</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.998</v>
+        <v>0.0051</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.0051</v>
-      </c>
-      <c r="G2" s="5" t="n">
         <v>0.0068</v>
       </c>
+      <c r="G2" s="5" t="inlineStr"/>
       <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr"/>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr"/>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr"/>
+      <c r="N2" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
+      <c r="O2" s="5" t="inlineStr"/>
       <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr"/>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr"/>
-      <c r="T2" s="5" t="inlineStr">
+      <c r="R2" s="5" t="inlineStr"/>
+      <c r="S2" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr"/>
-      <c r="V2" s="5" t="inlineStr">
+      <c r="T2" s="5" t="inlineStr"/>
+      <c r="U2" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr"/>
+      <c r="V2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1086,60 +1059,57 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.9473</v>
+        <v>0.9555</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.9555</v>
+        <v>0.9688</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.9611</v>
+        <v>0.007</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="G3" s="5" t="n">
         <v>0.0033</v>
       </c>
+      <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr"/>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr"/>
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
+      <c r="O3" s="5" t="inlineStr"/>
       <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr"/>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="W3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -1153,60 +1123,57 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.9199000000000001</v>
+        <v>0.9101</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.9101</v>
+        <v>0.9188</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.9125</v>
+        <v>0.013</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="G4" s="5" t="n">
         <v>0.0135</v>
       </c>
+      <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr"/>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr"/>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr"/>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr"/>
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr"/>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="T4" s="5" t="inlineStr"/>
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr"/>
+      <c r="V4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1220,56 +1187,53 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.8951</v>
+        <v>0.9224</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.9224</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>0.9324</v>
-      </c>
+        <v>0.9371</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
+      <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>25-26</t>
         </is>
       </c>
-      <c r="S5" s="5" t="inlineStr"/>
-      <c r="T5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr"/>
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>26-27</t>
         </is>
       </c>
-      <c r="U5" s="5" t="inlineStr"/>
-      <c r="V5" s="5" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr">
         <is>
           <t>27-28</t>
         </is>
       </c>
-      <c r="W5" s="5" t="inlineStr"/>
+      <c r="V5" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C5">
@@ -1302,9 +1266,9 @@
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="00F8696B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="0063BE7B"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
@@ -1502,18 +1466,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="V2:V5">
     <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W5">
-    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>